<commit_message>
docs(hw06): complete student extension root-cause analysis and finalize submission artifacts
</commit_message>
<xml_diff>
--- a/hw06/testcases/testcases-master.xlsx
+++ b/hw06/testcases/testcases-master.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>129 Logical Test Cases (43 per feature: 38 Reviewed AI + 5 Student Extensions)</t>
+          <t>129 Logical Test Cases (43 per feature: 38 Reviewed AI + 5 AI-assisted/student-selected extensions)</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -1419,7 +1419,7 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -4486,12 +4486,12 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N40" s="16" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -4563,12 +4563,12 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -4640,12 +4640,12 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N42" s="16" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N43" s="16" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
@@ -4794,12 +4794,12 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N44" s="16" t="inlineStr">
@@ -7600,7 +7600,7 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D83" s="15" t="inlineStr">
@@ -7645,12 +7645,12 @@
       </c>
       <c r="L83" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M83" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D84" s="15" t="inlineStr">
@@ -7722,12 +7722,12 @@
       </c>
       <c r="L84" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M84" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N84" s="16" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
@@ -7799,12 +7799,12 @@
       </c>
       <c r="L85" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M85" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D86" s="15" t="inlineStr">
@@ -7876,12 +7876,12 @@
       </c>
       <c r="L86" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M86" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N86" s="18" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D87" s="15" t="inlineStr">
@@ -7953,12 +7953,12 @@
       </c>
       <c r="L87" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M87" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D126" s="15" t="inlineStr">
@@ -10804,12 +10804,12 @@
       </c>
       <c r="L126" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M126" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N126" s="16" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D127" s="15" t="inlineStr">
@@ -10881,12 +10881,12 @@
       </c>
       <c r="L127" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M127" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N127" s="16" t="inlineStr">
@@ -10913,7 +10913,7 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D128" s="15" t="inlineStr">
@@ -10958,12 +10958,12 @@
       </c>
       <c r="L128" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M128" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N128" s="18" t="inlineStr">
@@ -10990,7 +10990,7 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D129" s="15" t="inlineStr">
@@ -11035,12 +11035,12 @@
       </c>
       <c r="L129" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M129" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N129" s="18" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D130" s="15" t="inlineStr">
@@ -11112,12 +11112,12 @@
       </c>
       <c r="L130" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M130" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N130" s="18" t="inlineStr">
@@ -11148,7 +11148,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -11157,7 +11157,7 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="25" customWidth="1" min="15" max="15"/>
@@ -14179,7 +14179,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -14224,12 +14224,12 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N40" s="16" t="inlineStr">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -14301,12 +14301,12 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
@@ -14333,7 +14333,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -14378,12 +14378,12 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N42" s="16" t="inlineStr">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
@@ -14455,12 +14455,12 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N43" s="16" t="inlineStr">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
@@ -14532,12 +14532,12 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N44" s="16" t="inlineStr">
@@ -14568,7 +14568,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -14577,7 +14577,7 @@
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="25" customWidth="1" min="15" max="15"/>
@@ -17447,7 +17447,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -17492,12 +17492,12 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N40" s="16" t="inlineStr">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -17569,12 +17569,12 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
@@ -17601,7 +17601,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -17646,12 +17646,12 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N42" s="16" t="inlineStr">
@@ -17678,7 +17678,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
@@ -17723,12 +17723,12 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N43" s="18" t="inlineStr">
@@ -17755,7 +17755,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
@@ -17800,12 +17800,12 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N44" s="16" t="inlineStr">
@@ -17836,7 +17836,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -17845,7 +17845,7 @@
     <col width="29" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
@@ -20715,7 +20715,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -20760,12 +20760,12 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N40" s="16" t="inlineStr">
@@ -20792,7 +20792,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -20837,12 +20837,12 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
@@ -20869,7 +20869,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -20914,12 +20914,12 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N42" s="18" t="inlineStr">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
@@ -20991,12 +20991,12 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N43" s="18" t="inlineStr">
@@ -21023,7 +21023,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Student Extension</t>
+          <t>AI-Assisted / Student-Selected Extension</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
@@ -21068,12 +21068,12 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>N/A (Student Authored)</t>
+          <t>N/A (AI-Assisted Extension)</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>Human authored extension exploring AI coverage gaps</t>
+          <t>AI-brainstormed idea selected by student; does not count as independently student-originated</t>
         </is>
       </c>
       <c r="N44" s="18" t="inlineStr">
@@ -21107,7 +21107,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21328,7 +21328,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Original Student Extension Cases Added</t>
+          <t>AI-Assisted / Student-Selected Extensions Added</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>15 independent student-original cases still required by PDF page 4</t>
         </is>
       </c>
     </row>

</xml_diff>